<commit_message>
Record Ender as payer of Idaho filing fee (joint account)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019wz211dBJ3nVUjGRBQudCu
</commit_message>
<xml_diff>
--- a/Digifender LLC (Idaho 2026)/04 Finance/Digifender Bookkeeping.xlsx
+++ b/Digifender LLC (Idaho 2026)/04 Finance/Digifender Bookkeeping.xlsx
@@ -2689,7 +2689,11 @@
       <c r="A6" s="24" t="n">
         <v>46324</v>
       </c>
-      <c r="B6" s="1" t="n"/>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Ender</t>
+        </is>
+      </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Idaho Secretary of State</t>
@@ -2697,7 +2701,7 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>Certificate of Organization filing fee, Digifender LLC (receipt 1410843). Card processor fees ($1.00 + 2.5%) are billed separately; add from card statement.</t>
+          <t>Certificate of Organization filing fee, Digifender LLC (receipt 1410843). Card processor fees ($1.00 + 2.5%) are billed separately; add from card statement. Paid by Ender from the owners' joint personal account (funds not split between members).</t>
         </is>
       </c>
       <c r="E6" s="22" t="n">

</xml_diff>